<commit_message>
Update database with complete author information; fix joblib path lookup to support root directory
</commit_message>
<xml_diff>
--- a/ML_FRC_BCJ_Vj_Database.xlsx
+++ b/ML_FRC_BCJ_Vj_Database.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kantekin\Desktop\FRC Paper\Code\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9BDD1B5-A15A-4AC2-92FE-0D4C9DF5CC61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6344B0C-9BE7-4337-9153-30E3A767F0DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="903" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -902,9 +902,6 @@
     <t>JHS6</t>
   </si>
   <si>
-    <t>Cui et al.</t>
-  </si>
-  <si>
     <t>SFNC-0-1</t>
   </si>
   <si>
@@ -920,9 +917,6 @@
     <t>SFCGC-50-1.5</t>
   </si>
   <si>
-    <t>Cai et al.</t>
-  </si>
-  <si>
     <t>ID</t>
   </si>
   <si>
@@ -936,6 +930,12 @@
   </si>
   <si>
     <t>fyv</t>
+  </si>
+  <si>
+    <t>Cai et al. (2024)</t>
+  </si>
+  <si>
+    <t>Cui et al. (2025)</t>
   </si>
 </sst>
 </file>
@@ -1067,10 +1067,10 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1388,7 +1388,7 @@
   <sheetData>
     <row r="1" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="B1" s="6" t="s">
         <v>183</v>
@@ -1418,7 +1418,7 @@
         <v>14</v>
       </c>
       <c r="K1" s="6" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="L1" s="6" t="s">
         <v>12</v>
@@ -1427,7 +1427,7 @@
         <v>13</v>
       </c>
       <c r="N1" s="6" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="O1" s="6" t="s">
         <v>261</v>
@@ -1451,14 +1451,14 @@
         <v>1</v>
       </c>
       <c r="V1" s="6" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
     </row>
     <row r="2" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A2" s="6">
         <v>1</v>
       </c>
-      <c r="B2" s="23" t="s">
+      <c r="B2" s="22" t="s">
         <v>184</v>
       </c>
       <c r="C2" s="6">
@@ -1526,7 +1526,7 @@
       <c r="A3" s="6">
         <v>2</v>
       </c>
-      <c r="B3" s="23"/>
+      <c r="B3" s="22"/>
       <c r="C3" s="6">
         <v>2</v>
       </c>
@@ -1592,7 +1592,7 @@
       <c r="A4" s="6">
         <v>3</v>
       </c>
-      <c r="B4" s="22" t="s">
+      <c r="B4" s="23" t="s">
         <v>209</v>
       </c>
       <c r="C4" s="14" t="s">
@@ -1660,7 +1660,7 @@
       <c r="A5" s="6">
         <v>4</v>
       </c>
-      <c r="B5" s="22"/>
+      <c r="B5" s="23"/>
       <c r="C5" s="14" t="s">
         <v>155</v>
       </c>
@@ -1726,7 +1726,7 @@
       <c r="A6" s="6">
         <v>5</v>
       </c>
-      <c r="B6" s="22"/>
+      <c r="B6" s="23"/>
       <c r="C6" s="14" t="s">
         <v>156</v>
       </c>
@@ -1792,7 +1792,7 @@
       <c r="A7" s="6">
         <v>6</v>
       </c>
-      <c r="B7" s="22"/>
+      <c r="B7" s="23"/>
       <c r="C7" s="14" t="s">
         <v>157</v>
       </c>
@@ -1858,7 +1858,7 @@
       <c r="A8" s="6">
         <v>7</v>
       </c>
-      <c r="B8" s="22" t="s">
+      <c r="B8" s="23" t="s">
         <v>208</v>
       </c>
       <c r="C8" s="6" t="s">
@@ -1926,7 +1926,7 @@
       <c r="A9" s="6">
         <v>8</v>
       </c>
-      <c r="B9" s="22"/>
+      <c r="B9" s="23"/>
       <c r="C9" s="6" t="s">
         <v>171</v>
       </c>
@@ -1992,7 +1992,7 @@
       <c r="A10" s="6">
         <v>9</v>
       </c>
-      <c r="B10" s="22" t="s">
+      <c r="B10" s="23" t="s">
         <v>210</v>
       </c>
       <c r="C10" s="6" t="s">
@@ -2060,7 +2060,7 @@
       <c r="A11" s="6">
         <v>10</v>
       </c>
-      <c r="B11" s="22"/>
+      <c r="B11" s="23"/>
       <c r="C11" s="6" t="s">
         <v>78</v>
       </c>
@@ -2126,7 +2126,7 @@
       <c r="A12" s="6">
         <v>11</v>
       </c>
-      <c r="B12" s="22"/>
+      <c r="B12" s="23"/>
       <c r="C12" s="6" t="s">
         <v>79</v>
       </c>
@@ -2192,7 +2192,7 @@
       <c r="A13" s="6">
         <v>12</v>
       </c>
-      <c r="B13" s="22"/>
+      <c r="B13" s="23"/>
       <c r="C13" s="6" t="s">
         <v>80</v>
       </c>
@@ -2258,7 +2258,7 @@
       <c r="A14" s="6">
         <v>13</v>
       </c>
-      <c r="B14" s="22"/>
+      <c r="B14" s="23"/>
       <c r="C14" s="6" t="s">
         <v>81</v>
       </c>
@@ -2324,7 +2324,7 @@
       <c r="A15" s="6">
         <v>14</v>
       </c>
-      <c r="B15" s="22"/>
+      <c r="B15" s="23"/>
       <c r="C15" s="6" t="s">
         <v>82</v>
       </c>
@@ -2390,7 +2390,7 @@
       <c r="A16" s="6">
         <v>15</v>
       </c>
-      <c r="B16" s="22" t="s">
+      <c r="B16" s="23" t="s">
         <v>211</v>
       </c>
       <c r="C16" s="6" t="s">
@@ -2458,7 +2458,7 @@
       <c r="A17" s="6">
         <v>16</v>
       </c>
-      <c r="B17" s="22"/>
+      <c r="B17" s="23"/>
       <c r="C17" s="6" t="s">
         <v>90</v>
       </c>
@@ -2524,7 +2524,7 @@
       <c r="A18" s="6">
         <v>17</v>
       </c>
-      <c r="B18" s="23" t="s">
+      <c r="B18" s="22" t="s">
         <v>185</v>
       </c>
       <c r="C18" s="6" t="s">
@@ -2592,7 +2592,7 @@
       <c r="A19" s="6">
         <v>18</v>
       </c>
-      <c r="B19" s="22"/>
+      <c r="B19" s="23"/>
       <c r="C19" s="6" t="s">
         <v>16</v>
       </c>
@@ -2658,7 +2658,7 @@
       <c r="A20" s="6">
         <v>19</v>
       </c>
-      <c r="B20" s="23" t="s">
+      <c r="B20" s="22" t="s">
         <v>186</v>
       </c>
       <c r="C20" s="6" t="s">
@@ -2726,7 +2726,7 @@
       <c r="A21" s="6">
         <v>20</v>
       </c>
-      <c r="B21" s="22"/>
+      <c r="B21" s="23"/>
       <c r="C21" s="6" t="s">
         <v>18</v>
       </c>
@@ -2792,7 +2792,7 @@
       <c r="A22" s="6">
         <v>21</v>
       </c>
-      <c r="B22" s="22"/>
+      <c r="B22" s="23"/>
       <c r="C22" s="6" t="s">
         <v>19</v>
       </c>
@@ -2858,7 +2858,7 @@
       <c r="A23" s="6">
         <v>22</v>
       </c>
-      <c r="B23" s="22"/>
+      <c r="B23" s="23"/>
       <c r="C23" s="6" t="s">
         <v>20</v>
       </c>
@@ -2924,7 +2924,7 @@
       <c r="A24" s="6">
         <v>23</v>
       </c>
-      <c r="B24" s="22"/>
+      <c r="B24" s="23"/>
       <c r="C24" s="6" t="s">
         <v>21</v>
       </c>
@@ -2990,7 +2990,7 @@
       <c r="A25" s="6">
         <v>24</v>
       </c>
-      <c r="B25" s="22"/>
+      <c r="B25" s="23"/>
       <c r="C25" s="6" t="s">
         <v>22</v>
       </c>
@@ -3056,7 +3056,7 @@
       <c r="A26" s="6">
         <v>25</v>
       </c>
-      <c r="B26" s="22"/>
+      <c r="B26" s="23"/>
       <c r="C26" s="6" t="s">
         <v>23</v>
       </c>
@@ -3122,7 +3122,7 @@
       <c r="A27" s="6">
         <v>26</v>
       </c>
-      <c r="B27" s="22"/>
+      <c r="B27" s="23"/>
       <c r="C27" s="6" t="s">
         <v>24</v>
       </c>
@@ -3188,7 +3188,7 @@
       <c r="A28" s="6">
         <v>27</v>
       </c>
-      <c r="B28" s="23" t="s">
+      <c r="B28" s="22" t="s">
         <v>187</v>
       </c>
       <c r="C28" s="6" t="s">
@@ -3256,7 +3256,7 @@
       <c r="A29" s="6">
         <v>28</v>
       </c>
-      <c r="B29" s="22"/>
+      <c r="B29" s="23"/>
       <c r="C29" s="6" t="s">
         <v>26</v>
       </c>
@@ -3390,7 +3390,7 @@
       <c r="A31" s="6">
         <v>30</v>
       </c>
-      <c r="B31" s="23" t="s">
+      <c r="B31" s="22" t="s">
         <v>189</v>
       </c>
       <c r="C31" s="6" t="s">
@@ -3458,7 +3458,7 @@
       <c r="A32" s="6">
         <v>31</v>
       </c>
-      <c r="B32" s="22"/>
+      <c r="B32" s="23"/>
       <c r="C32" s="6" t="s">
         <v>28</v>
       </c>
@@ -3524,7 +3524,7 @@
       <c r="A33" s="6">
         <v>32</v>
       </c>
-      <c r="B33" s="22"/>
+      <c r="B33" s="23"/>
       <c r="C33" s="6" t="s">
         <v>29</v>
       </c>
@@ -3590,7 +3590,7 @@
       <c r="A34" s="6">
         <v>33</v>
       </c>
-      <c r="B34" s="22"/>
+      <c r="B34" s="23"/>
       <c r="C34" s="6" t="s">
         <v>30</v>
       </c>
@@ -3656,7 +3656,7 @@
       <c r="A35" s="6">
         <v>34</v>
       </c>
-      <c r="B35" s="22"/>
+      <c r="B35" s="23"/>
       <c r="C35" s="6" t="s">
         <v>31</v>
       </c>
@@ -3722,7 +3722,7 @@
       <c r="A36" s="6">
         <v>35</v>
       </c>
-      <c r="B36" s="22"/>
+      <c r="B36" s="23"/>
       <c r="C36" s="6" t="s">
         <v>32</v>
       </c>
@@ -3856,7 +3856,7 @@
       <c r="A38" s="6">
         <v>37</v>
       </c>
-      <c r="B38" s="22" t="s">
+      <c r="B38" s="23" t="s">
         <v>241</v>
       </c>
       <c r="C38" s="6" t="s">
@@ -3924,7 +3924,7 @@
       <c r="A39" s="6">
         <v>38</v>
       </c>
-      <c r="B39" s="22"/>
+      <c r="B39" s="23"/>
       <c r="C39" s="6" t="s">
         <v>243</v>
       </c>
@@ -4058,7 +4058,7 @@
       <c r="A41" s="6">
         <v>40</v>
       </c>
-      <c r="B41" s="22" t="s">
+      <c r="B41" s="23" t="s">
         <v>192</v>
       </c>
       <c r="C41" s="6" t="s">
@@ -4126,7 +4126,7 @@
       <c r="A42" s="6">
         <v>41</v>
       </c>
-      <c r="B42" s="22"/>
+      <c r="B42" s="23"/>
       <c r="C42" s="6" t="s">
         <v>28</v>
       </c>
@@ -4192,7 +4192,7 @@
       <c r="A43" s="6">
         <v>42</v>
       </c>
-      <c r="B43" s="22"/>
+      <c r="B43" s="23"/>
       <c r="C43" s="6" t="s">
         <v>168</v>
       </c>
@@ -4258,7 +4258,7 @@
       <c r="A44" s="6">
         <v>43</v>
       </c>
-      <c r="B44" s="23" t="s">
+      <c r="B44" s="22" t="s">
         <v>193</v>
       </c>
       <c r="C44" s="6" t="s">
@@ -4326,7 +4326,7 @@
       <c r="A45" s="6">
         <v>44</v>
       </c>
-      <c r="B45" s="22"/>
+      <c r="B45" s="23"/>
       <c r="C45" s="6" t="s">
         <v>34</v>
       </c>
@@ -4392,7 +4392,7 @@
       <c r="A46" s="6">
         <v>45</v>
       </c>
-      <c r="B46" s="22"/>
+      <c r="B46" s="23"/>
       <c r="C46" s="6" t="s">
         <v>35</v>
       </c>
@@ -4458,7 +4458,7 @@
       <c r="A47" s="6">
         <v>46</v>
       </c>
-      <c r="B47" s="22"/>
+      <c r="B47" s="23"/>
       <c r="C47" s="6" t="s">
         <v>36</v>
       </c>
@@ -4592,7 +4592,7 @@
       <c r="A49" s="6">
         <v>48</v>
       </c>
-      <c r="B49" s="22" t="s">
+      <c r="B49" s="23" t="s">
         <v>195</v>
       </c>
       <c r="C49" s="6" t="s">
@@ -4660,7 +4660,7 @@
       <c r="A50" s="6">
         <v>49</v>
       </c>
-      <c r="B50" s="22"/>
+      <c r="B50" s="23"/>
       <c r="C50" s="6" t="s">
         <v>39</v>
       </c>
@@ -4726,7 +4726,7 @@
       <c r="A51" s="6">
         <v>50</v>
       </c>
-      <c r="B51" s="22"/>
+      <c r="B51" s="23"/>
       <c r="C51" s="6" t="s">
         <v>40</v>
       </c>
@@ -4792,7 +4792,7 @@
       <c r="A52" s="6">
         <v>51</v>
       </c>
-      <c r="B52" s="22" t="s">
+      <c r="B52" s="23" t="s">
         <v>196</v>
       </c>
       <c r="C52" s="6" t="s">
@@ -4860,7 +4860,7 @@
       <c r="A53" s="6">
         <v>52</v>
       </c>
-      <c r="B53" s="22"/>
+      <c r="B53" s="23"/>
       <c r="C53" s="6" t="s">
         <v>42</v>
       </c>
@@ -4926,7 +4926,7 @@
       <c r="A54" s="6">
         <v>53</v>
       </c>
-      <c r="B54" s="22"/>
+      <c r="B54" s="23"/>
       <c r="C54" s="6" t="s">
         <v>43</v>
       </c>
@@ -4992,7 +4992,7 @@
       <c r="A55" s="6">
         <v>54</v>
       </c>
-      <c r="B55" s="22"/>
+      <c r="B55" s="23"/>
       <c r="C55" s="6" t="s">
         <v>44</v>
       </c>
@@ -5058,7 +5058,7 @@
       <c r="A56" s="6">
         <v>55</v>
       </c>
-      <c r="B56" s="22"/>
+      <c r="B56" s="23"/>
       <c r="C56" s="6" t="s">
         <v>45</v>
       </c>
@@ -5124,7 +5124,7 @@
       <c r="A57" s="6">
         <v>56</v>
       </c>
-      <c r="B57" s="22"/>
+      <c r="B57" s="23"/>
       <c r="C57" s="6" t="s">
         <v>46</v>
       </c>
@@ -5190,7 +5190,7 @@
       <c r="A58" s="6">
         <v>57</v>
       </c>
-      <c r="B58" s="22"/>
+      <c r="B58" s="23"/>
       <c r="C58" s="6" t="s">
         <v>47</v>
       </c>
@@ -5256,7 +5256,7 @@
       <c r="A59" s="6">
         <v>58</v>
       </c>
-      <c r="B59" s="22" t="s">
+      <c r="B59" s="23" t="s">
         <v>197</v>
       </c>
       <c r="C59" s="6">
@@ -5324,7 +5324,7 @@
       <c r="A60" s="6">
         <v>59</v>
       </c>
-      <c r="B60" s="22"/>
+      <c r="B60" s="23"/>
       <c r="C60" s="6">
         <v>3</v>
       </c>
@@ -5390,7 +5390,7 @@
       <c r="A61" s="6">
         <v>60</v>
       </c>
-      <c r="B61" s="22"/>
+      <c r="B61" s="23"/>
       <c r="C61" s="6">
         <v>4</v>
       </c>
@@ -5456,7 +5456,7 @@
       <c r="A62" s="6">
         <v>61</v>
       </c>
-      <c r="B62" s="22" t="s">
+      <c r="B62" s="23" t="s">
         <v>198</v>
       </c>
       <c r="C62" s="6" t="s">
@@ -5524,7 +5524,7 @@
       <c r="A63" s="6">
         <v>62</v>
       </c>
-      <c r="B63" s="22"/>
+      <c r="B63" s="23"/>
       <c r="C63" s="6" t="s">
         <v>50</v>
       </c>
@@ -5590,7 +5590,7 @@
       <c r="A64" s="6">
         <v>63</v>
       </c>
-      <c r="B64" s="22"/>
+      <c r="B64" s="23"/>
       <c r="C64" s="6" t="s">
         <v>51</v>
       </c>
@@ -5656,7 +5656,7 @@
       <c r="A65" s="6">
         <v>64</v>
       </c>
-      <c r="B65" s="22"/>
+      <c r="B65" s="23"/>
       <c r="C65" s="6" t="s">
         <v>49</v>
       </c>
@@ -5722,7 +5722,7 @@
       <c r="A66" s="6">
         <v>65</v>
       </c>
-      <c r="B66" s="22" t="s">
+      <c r="B66" s="23" t="s">
         <v>199</v>
       </c>
       <c r="C66" s="6" t="s">
@@ -5790,7 +5790,7 @@
       <c r="A67" s="6">
         <v>66</v>
       </c>
-      <c r="B67" s="22"/>
+      <c r="B67" s="23"/>
       <c r="C67" s="6" t="s">
         <v>53</v>
       </c>
@@ -5856,7 +5856,7 @@
       <c r="A68" s="6">
         <v>67</v>
       </c>
-      <c r="B68" s="22"/>
+      <c r="B68" s="23"/>
       <c r="C68" s="6" t="s">
         <v>54</v>
       </c>
@@ -5922,7 +5922,7 @@
       <c r="A69" s="6">
         <v>68</v>
       </c>
-      <c r="B69" s="22"/>
+      <c r="B69" s="23"/>
       <c r="C69" s="6" t="s">
         <v>55</v>
       </c>
@@ -5988,7 +5988,7 @@
       <c r="A70" s="6">
         <v>69</v>
       </c>
-      <c r="B70" s="22"/>
+      <c r="B70" s="23"/>
       <c r="C70" s="6" t="s">
         <v>56</v>
       </c>
@@ -6054,7 +6054,7 @@
       <c r="A71" s="6">
         <v>70</v>
       </c>
-      <c r="B71" s="22"/>
+      <c r="B71" s="23"/>
       <c r="C71" s="6" t="s">
         <v>57</v>
       </c>
@@ -6256,7 +6256,7 @@
       <c r="A74" s="6">
         <v>73</v>
       </c>
-      <c r="B74" s="22" t="s">
+      <c r="B74" s="23" t="s">
         <v>201</v>
       </c>
       <c r="C74" s="6" t="s">
@@ -6324,7 +6324,7 @@
       <c r="A75" s="6">
         <v>74</v>
       </c>
-      <c r="B75" s="22"/>
+      <c r="B75" s="23"/>
       <c r="C75" s="6" t="s">
         <v>60</v>
       </c>
@@ -6526,7 +6526,7 @@
       <c r="A78" s="6">
         <v>77</v>
       </c>
-      <c r="B78" s="22" t="s">
+      <c r="B78" s="23" t="s">
         <v>204</v>
       </c>
       <c r="C78" s="6" t="s">
@@ -6594,7 +6594,7 @@
       <c r="A79" s="6">
         <v>78</v>
       </c>
-      <c r="B79" s="22"/>
+      <c r="B79" s="23"/>
       <c r="C79" s="6" t="s">
         <v>63</v>
       </c>
@@ -6660,7 +6660,7 @@
       <c r="A80" s="6">
         <v>79</v>
       </c>
-      <c r="B80" s="22"/>
+      <c r="B80" s="23"/>
       <c r="C80" s="6" t="s">
         <v>64</v>
       </c>
@@ -6726,7 +6726,7 @@
       <c r="A81" s="6">
         <v>80</v>
       </c>
-      <c r="B81" s="22"/>
+      <c r="B81" s="23"/>
       <c r="C81" s="6" t="s">
         <v>65</v>
       </c>
@@ -6792,7 +6792,7 @@
       <c r="A82" s="6">
         <v>81</v>
       </c>
-      <c r="B82" s="22" t="s">
+      <c r="B82" s="23" t="s">
         <v>205</v>
       </c>
       <c r="C82" s="6" t="s">
@@ -6860,7 +6860,7 @@
       <c r="A83" s="6">
         <v>82</v>
       </c>
-      <c r="B83" s="22"/>
+      <c r="B83" s="23"/>
       <c r="C83" s="6" t="s">
         <v>67</v>
       </c>
@@ -6926,7 +6926,7 @@
       <c r="A84" s="6">
         <v>83</v>
       </c>
-      <c r="B84" s="22" t="s">
+      <c r="B84" s="23" t="s">
         <v>206</v>
       </c>
       <c r="C84" s="6" t="s">
@@ -6994,7 +6994,7 @@
       <c r="A85" s="6">
         <v>84</v>
       </c>
-      <c r="B85" s="22"/>
+      <c r="B85" s="23"/>
       <c r="C85" s="6" t="s">
         <v>69</v>
       </c>
@@ -7060,7 +7060,7 @@
       <c r="A86" s="6">
         <v>85</v>
       </c>
-      <c r="B86" s="22" t="s">
+      <c r="B86" s="23" t="s">
         <v>207</v>
       </c>
       <c r="C86" s="6" t="s">
@@ -7128,7 +7128,7 @@
       <c r="A87" s="6">
         <v>86</v>
       </c>
-      <c r="B87" s="22"/>
+      <c r="B87" s="23"/>
       <c r="C87" s="6" t="s">
         <v>71</v>
       </c>
@@ -7194,7 +7194,7 @@
       <c r="A88" s="6">
         <v>87</v>
       </c>
-      <c r="B88" s="22"/>
+      <c r="B88" s="23"/>
       <c r="C88" s="6" t="s">
         <v>72</v>
       </c>
@@ -7260,7 +7260,7 @@
       <c r="A89" s="6">
         <v>88</v>
       </c>
-      <c r="B89" s="22"/>
+      <c r="B89" s="23"/>
       <c r="C89" s="6" t="s">
         <v>73</v>
       </c>
@@ -7326,7 +7326,7 @@
       <c r="A90" s="6">
         <v>89</v>
       </c>
-      <c r="B90" s="22" t="s">
+      <c r="B90" s="23" t="s">
         <v>217</v>
       </c>
       <c r="C90" s="6">
@@ -7394,7 +7394,7 @@
       <c r="A91" s="6">
         <v>90</v>
       </c>
-      <c r="B91" s="22"/>
+      <c r="B91" s="23"/>
       <c r="C91" s="6">
         <v>5</v>
       </c>
@@ -7460,7 +7460,7 @@
       <c r="A92" s="6">
         <v>91</v>
       </c>
-      <c r="B92" s="22"/>
+      <c r="B92" s="23"/>
       <c r="C92" s="6">
         <v>6</v>
       </c>
@@ -7526,7 +7526,7 @@
       <c r="A93" s="6">
         <v>92</v>
       </c>
-      <c r="B93" s="22"/>
+      <c r="B93" s="23"/>
       <c r="C93" s="6">
         <v>8</v>
       </c>
@@ -7592,7 +7592,7 @@
       <c r="A94" s="6">
         <v>93</v>
       </c>
-      <c r="B94" s="22"/>
+      <c r="B94" s="23"/>
       <c r="C94" s="6">
         <v>9</v>
       </c>
@@ -7658,7 +7658,7 @@
       <c r="A95" s="6">
         <v>94</v>
       </c>
-      <c r="B95" s="22"/>
+      <c r="B95" s="23"/>
       <c r="C95" s="6">
         <v>10</v>
       </c>
@@ -7724,7 +7724,7 @@
       <c r="A96" s="6">
         <v>95</v>
       </c>
-      <c r="B96" s="22" t="s">
+      <c r="B96" s="23" t="s">
         <v>256</v>
       </c>
       <c r="C96" s="6" t="s">
@@ -7792,7 +7792,7 @@
       <c r="A97" s="6">
         <v>96</v>
       </c>
-      <c r="B97" s="22"/>
+      <c r="B97" s="23"/>
       <c r="C97" s="6" t="s">
         <v>258</v>
       </c>
@@ -7858,7 +7858,7 @@
       <c r="A98" s="6">
         <v>97</v>
       </c>
-      <c r="B98" s="22"/>
+      <c r="B98" s="23"/>
       <c r="C98" s="6" t="s">
         <v>259</v>
       </c>
@@ -7924,7 +7924,7 @@
       <c r="A99" s="6">
         <v>98</v>
       </c>
-      <c r="B99" s="23" t="s">
+      <c r="B99" s="22" t="s">
         <v>218</v>
       </c>
       <c r="C99" s="14" t="s">
@@ -7992,7 +7992,7 @@
       <c r="A100" s="6">
         <v>99</v>
       </c>
-      <c r="B100" s="23"/>
+      <c r="B100" s="22"/>
       <c r="C100" s="14" t="s">
         <v>60</v>
       </c>
@@ -8058,7 +8058,7 @@
       <c r="A101" s="6">
         <v>100</v>
       </c>
-      <c r="B101" s="23"/>
+      <c r="B101" s="22"/>
       <c r="C101" s="14" t="s">
         <v>159</v>
       </c>
@@ -8124,7 +8124,7 @@
       <c r="A102" s="6">
         <v>101</v>
       </c>
-      <c r="B102" s="23"/>
+      <c r="B102" s="22"/>
       <c r="C102" s="14" t="s">
         <v>160</v>
       </c>
@@ -8190,7 +8190,7 @@
       <c r="A103" s="6">
         <v>102</v>
       </c>
-      <c r="B103" s="22" t="s">
+      <c r="B103" s="23" t="s">
         <v>255</v>
       </c>
       <c r="C103" s="6" t="s">
@@ -8258,7 +8258,7 @@
       <c r="A104" s="6">
         <v>103</v>
       </c>
-      <c r="B104" s="22"/>
+      <c r="B104" s="23"/>
       <c r="C104" s="6" t="s">
         <v>245</v>
       </c>
@@ -8324,7 +8324,7 @@
       <c r="A105" s="6">
         <v>104</v>
       </c>
-      <c r="B105" s="22" t="s">
+      <c r="B105" s="23" t="s">
         <v>219</v>
       </c>
       <c r="C105" s="6" t="s">
@@ -8392,7 +8392,7 @@
       <c r="A106" s="6">
         <v>105</v>
       </c>
-      <c r="B106" s="22"/>
+      <c r="B106" s="23"/>
       <c r="C106" s="6" t="s">
         <v>75</v>
       </c>
@@ -8458,7 +8458,7 @@
       <c r="A107" s="6">
         <v>106</v>
       </c>
-      <c r="B107" s="22"/>
+      <c r="B107" s="23"/>
       <c r="C107" s="6" t="s">
         <v>76</v>
       </c>
@@ -8524,7 +8524,7 @@
       <c r="A108" s="6">
         <v>107</v>
       </c>
-      <c r="B108" s="22" t="s">
+      <c r="B108" s="23" t="s">
         <v>235</v>
       </c>
       <c r="C108" s="6" t="s">
@@ -8592,7 +8592,7 @@
       <c r="A109" s="6">
         <v>108</v>
       </c>
-      <c r="B109" s="22"/>
+      <c r="B109" s="23"/>
       <c r="C109" s="6" t="s">
         <v>237</v>
       </c>
@@ -8658,7 +8658,7 @@
       <c r="A110" s="6">
         <v>109</v>
       </c>
-      <c r="B110" s="22"/>
+      <c r="B110" s="23"/>
       <c r="C110" s="6" t="s">
         <v>238</v>
       </c>
@@ -8724,7 +8724,7 @@
       <c r="A111" s="6">
         <v>110</v>
       </c>
-      <c r="B111" s="22"/>
+      <c r="B111" s="23"/>
       <c r="C111" s="6" t="s">
         <v>239</v>
       </c>
@@ -8790,7 +8790,7 @@
       <c r="A112" s="6">
         <v>111</v>
       </c>
-      <c r="B112" s="22" t="s">
+      <c r="B112" s="23" t="s">
         <v>221</v>
       </c>
       <c r="C112" s="6" t="s">
@@ -8858,7 +8858,7 @@
       <c r="A113" s="6">
         <v>112</v>
       </c>
-      <c r="B113" s="22"/>
+      <c r="B113" s="23"/>
       <c r="C113" s="6" t="s">
         <v>84</v>
       </c>
@@ -8924,7 +8924,7 @@
       <c r="A114" s="6">
         <v>113</v>
       </c>
-      <c r="B114" s="22" t="s">
+      <c r="B114" s="23" t="s">
         <v>222</v>
       </c>
       <c r="C114" s="6" t="s">
@@ -8992,7 +8992,7 @@
       <c r="A115" s="6">
         <v>114</v>
       </c>
-      <c r="B115" s="22"/>
+      <c r="B115" s="23"/>
       <c r="C115" s="6" t="s">
         <v>86</v>
       </c>
@@ -9058,7 +9058,7 @@
       <c r="A116" s="6">
         <v>115</v>
       </c>
-      <c r="B116" s="22"/>
+      <c r="B116" s="23"/>
       <c r="C116" s="6" t="s">
         <v>87</v>
       </c>
@@ -9124,7 +9124,7 @@
       <c r="A117" s="6">
         <v>116</v>
       </c>
-      <c r="B117" s="22"/>
+      <c r="B117" s="23"/>
       <c r="C117" s="6" t="s">
         <v>88</v>
       </c>
@@ -9190,7 +9190,7 @@
       <c r="A118" s="6">
         <v>117</v>
       </c>
-      <c r="B118" s="23" t="s">
+      <c r="B118" s="22" t="s">
         <v>223</v>
       </c>
       <c r="C118" s="14" t="s">
@@ -9258,7 +9258,7 @@
       <c r="A119" s="6">
         <v>118</v>
       </c>
-      <c r="B119" s="23"/>
+      <c r="B119" s="22"/>
       <c r="C119" s="14" t="s">
         <v>140</v>
       </c>
@@ -9324,7 +9324,7 @@
       <c r="A120" s="6">
         <v>119</v>
       </c>
-      <c r="B120" s="23"/>
+      <c r="B120" s="22"/>
       <c r="C120" s="14" t="s">
         <v>141</v>
       </c>
@@ -9390,7 +9390,7 @@
       <c r="A121" s="6">
         <v>120</v>
       </c>
-      <c r="B121" s="23"/>
+      <c r="B121" s="22"/>
       <c r="C121" s="14" t="s">
         <v>142</v>
       </c>
@@ -9456,7 +9456,7 @@
       <c r="A122" s="6">
         <v>121</v>
       </c>
-      <c r="B122" s="23"/>
+      <c r="B122" s="22"/>
       <c r="C122" s="14" t="s">
         <v>260</v>
       </c>
@@ -9522,7 +9522,7 @@
       <c r="A123" s="6">
         <v>122</v>
       </c>
-      <c r="B123" s="23"/>
+      <c r="B123" s="22"/>
       <c r="C123" s="14" t="s">
         <v>143</v>
       </c>
@@ -9588,7 +9588,7 @@
       <c r="A124" s="6">
         <v>123</v>
       </c>
-      <c r="B124" s="23"/>
+      <c r="B124" s="22"/>
       <c r="C124" s="14" t="s">
         <v>144</v>
       </c>
@@ -9654,7 +9654,7 @@
       <c r="A125" s="6">
         <v>124</v>
       </c>
-      <c r="B125" s="23"/>
+      <c r="B125" s="22"/>
       <c r="C125" s="14" t="s">
         <v>145</v>
       </c>
@@ -9720,7 +9720,7 @@
       <c r="A126" s="6">
         <v>125</v>
       </c>
-      <c r="B126" s="23" t="s">
+      <c r="B126" s="22" t="s">
         <v>224</v>
       </c>
       <c r="C126" s="14" t="s">
@@ -9788,7 +9788,7 @@
       <c r="A127" s="6">
         <v>126</v>
       </c>
-      <c r="B127" s="23"/>
+      <c r="B127" s="22"/>
       <c r="C127" s="14" t="s">
         <v>147</v>
       </c>
@@ -9854,7 +9854,7 @@
       <c r="A128" s="6">
         <v>127</v>
       </c>
-      <c r="B128" s="23"/>
+      <c r="B128" s="22"/>
       <c r="C128" s="14" t="s">
         <v>148</v>
       </c>
@@ -9920,7 +9920,7 @@
       <c r="A129" s="6">
         <v>128</v>
       </c>
-      <c r="B129" s="23"/>
+      <c r="B129" s="22"/>
       <c r="C129" s="14" t="s">
         <v>149</v>
       </c>
@@ -9986,7 +9986,7 @@
       <c r="A130" s="6">
         <v>129</v>
       </c>
-      <c r="B130" s="23"/>
+      <c r="B130" s="22"/>
       <c r="C130" s="14" t="s">
         <v>150</v>
       </c>
@@ -10052,7 +10052,7 @@
       <c r="A131" s="6">
         <v>130</v>
       </c>
-      <c r="B131" s="23"/>
+      <c r="B131" s="22"/>
       <c r="C131" s="14" t="s">
         <v>151</v>
       </c>
@@ -10254,7 +10254,7 @@
       <c r="A134" s="6">
         <v>133</v>
       </c>
-      <c r="B134" s="23" t="s">
+      <c r="B134" s="22" t="s">
         <v>227</v>
       </c>
       <c r="C134" s="14" t="s">
@@ -10322,7 +10322,7 @@
       <c r="A135" s="6">
         <v>134</v>
       </c>
-      <c r="B135" s="23"/>
+      <c r="B135" s="22"/>
       <c r="C135" s="14" t="s">
         <v>162</v>
       </c>
@@ -10388,7 +10388,7 @@
       <c r="A136" s="6">
         <v>135</v>
       </c>
-      <c r="B136" s="23"/>
+      <c r="B136" s="22"/>
       <c r="C136" s="14" t="s">
         <v>163</v>
       </c>
@@ -10454,7 +10454,7 @@
       <c r="A137" s="6">
         <v>136</v>
       </c>
-      <c r="B137" s="23"/>
+      <c r="B137" s="22"/>
       <c r="C137" s="14" t="s">
         <v>164</v>
       </c>
@@ -10520,7 +10520,7 @@
       <c r="A138" s="6">
         <v>137</v>
       </c>
-      <c r="B138" s="23"/>
+      <c r="B138" s="22"/>
       <c r="C138" s="14" t="s">
         <v>165</v>
       </c>
@@ -10586,7 +10586,7 @@
       <c r="A139" s="6">
         <v>138</v>
       </c>
-      <c r="B139" s="22" t="s">
+      <c r="B139" s="23" t="s">
         <v>228</v>
       </c>
       <c r="C139" s="6" t="s">
@@ -10654,7 +10654,7 @@
       <c r="A140" s="6">
         <v>139</v>
       </c>
-      <c r="B140" s="22"/>
+      <c r="B140" s="23"/>
       <c r="C140" s="6" t="s">
         <v>115</v>
       </c>
@@ -10720,8 +10720,8 @@
       <c r="A141" s="6">
         <v>140</v>
       </c>
-      <c r="B141" s="22" t="s">
-        <v>294</v>
+      <c r="B141" s="23" t="s">
+        <v>292</v>
       </c>
       <c r="C141" s="6" t="s">
         <v>116</v>
@@ -10788,7 +10788,7 @@
       <c r="A142" s="6">
         <v>141</v>
       </c>
-      <c r="B142" s="22"/>
+      <c r="B142" s="23"/>
       <c r="C142" s="6" t="s">
         <v>117</v>
       </c>
@@ -10854,7 +10854,7 @@
       <c r="A143" s="6">
         <v>142</v>
       </c>
-      <c r="B143" s="22"/>
+      <c r="B143" s="23"/>
       <c r="C143" s="6" t="s">
         <v>118</v>
       </c>
@@ -10920,7 +10920,7 @@
       <c r="A144" s="6">
         <v>143</v>
       </c>
-      <c r="B144" s="22"/>
+      <c r="B144" s="23"/>
       <c r="C144" s="6" t="s">
         <v>119</v>
       </c>
@@ -10986,7 +10986,7 @@
       <c r="A145" s="6">
         <v>144</v>
       </c>
-      <c r="B145" s="22"/>
+      <c r="B145" s="23"/>
       <c r="C145" s="6" t="s">
         <v>120</v>
       </c>
@@ -11052,7 +11052,7 @@
       <c r="A146" s="6">
         <v>145</v>
       </c>
-      <c r="B146" s="22"/>
+      <c r="B146" s="23"/>
       <c r="C146" s="6" t="s">
         <v>121</v>
       </c>
@@ -11118,7 +11118,7 @@
       <c r="A147" s="6">
         <v>146</v>
       </c>
-      <c r="B147" s="22" t="s">
+      <c r="B147" s="23" t="s">
         <v>229</v>
       </c>
       <c r="C147" s="6" t="s">
@@ -11186,7 +11186,7 @@
       <c r="A148" s="6">
         <v>147</v>
       </c>
-      <c r="B148" s="22"/>
+      <c r="B148" s="23"/>
       <c r="C148" s="6" t="s">
         <v>123</v>
       </c>
@@ -11252,7 +11252,7 @@
       <c r="A149" s="6">
         <v>148</v>
       </c>
-      <c r="B149" s="22"/>
+      <c r="B149" s="23"/>
       <c r="C149" s="6" t="s">
         <v>124</v>
       </c>
@@ -11318,7 +11318,7 @@
       <c r="A150" s="6">
         <v>149</v>
       </c>
-      <c r="B150" s="22"/>
+      <c r="B150" s="23"/>
       <c r="C150" s="6" t="s">
         <v>125</v>
       </c>
@@ -11384,7 +11384,7 @@
       <c r="A151" s="6">
         <v>150</v>
       </c>
-      <c r="B151" s="22"/>
+      <c r="B151" s="23"/>
       <c r="C151" s="6" t="s">
         <v>126</v>
       </c>
@@ -11450,7 +11450,7 @@
       <c r="A152" s="6">
         <v>151</v>
       </c>
-      <c r="B152" s="22" t="s">
+      <c r="B152" s="23" t="s">
         <v>230</v>
       </c>
       <c r="C152" s="6" t="s">
@@ -11518,7 +11518,7 @@
       <c r="A153" s="6">
         <v>152</v>
       </c>
-      <c r="B153" s="22"/>
+      <c r="B153" s="23"/>
       <c r="C153" s="6" t="s">
         <v>128</v>
       </c>
@@ -11584,7 +11584,7 @@
       <c r="A154" s="6">
         <v>153</v>
       </c>
-      <c r="B154" s="22"/>
+      <c r="B154" s="23"/>
       <c r="C154" s="14" t="s">
         <v>138</v>
       </c>
@@ -11650,7 +11650,7 @@
       <c r="A155" s="6">
         <v>154</v>
       </c>
-      <c r="B155" s="22" t="s">
+      <c r="B155" s="23" t="s">
         <v>231</v>
       </c>
       <c r="C155" s="6" t="s">
@@ -11718,7 +11718,7 @@
       <c r="A156" s="6">
         <v>155</v>
       </c>
-      <c r="B156" s="22"/>
+      <c r="B156" s="23"/>
       <c r="C156" s="6" t="s">
         <v>173</v>
       </c>
@@ -11784,7 +11784,7 @@
       <c r="A157" s="6">
         <v>156</v>
       </c>
-      <c r="B157" s="22"/>
+      <c r="B157" s="23"/>
       <c r="C157" s="6" t="s">
         <v>174</v>
       </c>
@@ -11850,7 +11850,7 @@
       <c r="A158" s="6">
         <v>157</v>
       </c>
-      <c r="B158" s="22"/>
+      <c r="B158" s="23"/>
       <c r="C158" s="6" t="s">
         <v>175</v>
       </c>
@@ -11916,7 +11916,7 @@
       <c r="A159" s="6">
         <v>158</v>
       </c>
-      <c r="B159" s="22"/>
+      <c r="B159" s="23"/>
       <c r="C159" s="6" t="s">
         <v>176</v>
       </c>
@@ -11982,7 +11982,7 @@
       <c r="A160" s="6">
         <v>159</v>
       </c>
-      <c r="B160" s="22"/>
+      <c r="B160" s="23"/>
       <c r="C160" s="6" t="s">
         <v>177</v>
       </c>
@@ -12048,7 +12048,7 @@
       <c r="A161" s="6">
         <v>160</v>
       </c>
-      <c r="B161" s="22"/>
+      <c r="B161" s="23"/>
       <c r="C161" s="6" t="s">
         <v>178</v>
       </c>
@@ -12182,7 +12182,7 @@
       <c r="A163" s="6">
         <v>162</v>
       </c>
-      <c r="B163" s="22" t="s">
+      <c r="B163" s="23" t="s">
         <v>240</v>
       </c>
       <c r="C163" s="6" t="s">
@@ -12250,7 +12250,7 @@
       <c r="A164" s="6">
         <v>163</v>
       </c>
-      <c r="B164" s="22"/>
+      <c r="B164" s="23"/>
       <c r="C164" s="6" t="s">
         <v>263</v>
       </c>
@@ -12316,7 +12316,7 @@
       <c r="A165" s="6">
         <v>164</v>
       </c>
-      <c r="B165" s="22"/>
+      <c r="B165" s="23"/>
       <c r="C165" s="6" t="s">
         <v>264</v>
       </c>
@@ -12382,7 +12382,7 @@
       <c r="A166" s="6">
         <v>165</v>
       </c>
-      <c r="B166" s="22"/>
+      <c r="B166" s="23"/>
       <c r="C166" s="6" t="s">
         <v>265</v>
       </c>
@@ -12448,7 +12448,7 @@
       <c r="A167" s="6">
         <v>166</v>
       </c>
-      <c r="B167" s="22"/>
+      <c r="B167" s="23"/>
       <c r="C167" s="6" t="s">
         <v>266</v>
       </c>
@@ -12514,7 +12514,7 @@
       <c r="A168" s="6">
         <v>167</v>
       </c>
-      <c r="B168" s="22"/>
+      <c r="B168" s="23"/>
       <c r="C168" s="6" t="s">
         <v>267</v>
       </c>
@@ -12580,7 +12580,7 @@
       <c r="A169" s="6">
         <v>168</v>
       </c>
-      <c r="B169" s="22"/>
+      <c r="B169" s="23"/>
       <c r="C169" s="6" t="s">
         <v>268</v>
       </c>
@@ -12646,7 +12646,7 @@
       <c r="A170" s="6">
         <v>169</v>
       </c>
-      <c r="B170" s="22" t="s">
+      <c r="B170" s="23" t="s">
         <v>272</v>
       </c>
       <c r="C170" s="6" t="s">
@@ -12714,7 +12714,7 @@
       <c r="A171" s="6">
         <v>170</v>
       </c>
-      <c r="B171" s="22"/>
+      <c r="B171" s="23"/>
       <c r="C171" s="6" t="s">
         <v>270</v>
       </c>
@@ -12780,7 +12780,7 @@
       <c r="A172" s="6">
         <v>171</v>
       </c>
-      <c r="B172" s="22"/>
+      <c r="B172" s="23"/>
       <c r="C172" s="6" t="s">
         <v>271</v>
       </c>
@@ -12846,7 +12846,7 @@
       <c r="A173" s="6">
         <v>172</v>
       </c>
-      <c r="B173" s="22" t="s">
+      <c r="B173" s="23" t="s">
         <v>278</v>
       </c>
       <c r="C173" s="6" t="s">
@@ -12914,7 +12914,7 @@
       <c r="A174" s="6">
         <v>173</v>
       </c>
-      <c r="B174" s="22"/>
+      <c r="B174" s="23"/>
       <c r="C174" s="6" t="s">
         <v>274</v>
       </c>
@@ -12980,7 +12980,7 @@
       <c r="A175" s="6">
         <v>174</v>
       </c>
-      <c r="B175" s="22"/>
+      <c r="B175" s="23"/>
       <c r="C175" s="6" t="s">
         <v>275</v>
       </c>
@@ -13046,7 +13046,7 @@
       <c r="A176" s="6">
         <v>175</v>
       </c>
-      <c r="B176" s="22"/>
+      <c r="B176" s="23"/>
       <c r="C176" s="6" t="s">
         <v>276</v>
       </c>
@@ -13112,7 +13112,7 @@
       <c r="A177" s="6">
         <v>176</v>
       </c>
-      <c r="B177" s="22"/>
+      <c r="B177" s="23"/>
       <c r="C177" s="6" t="s">
         <v>277</v>
       </c>
@@ -13178,8 +13178,8 @@
       <c r="A178" s="6">
         <v>177</v>
       </c>
-      <c r="B178" s="22" t="s">
-        <v>285</v>
+      <c r="B178" s="23" t="s">
+        <v>296</v>
       </c>
       <c r="C178" s="6" t="s">
         <v>279</v>
@@ -13246,7 +13246,7 @@
       <c r="A179" s="6">
         <v>178</v>
       </c>
-      <c r="B179" s="22"/>
+      <c r="B179" s="23"/>
       <c r="C179" s="6" t="s">
         <v>280</v>
       </c>
@@ -13312,7 +13312,7 @@
       <c r="A180" s="6">
         <v>179</v>
       </c>
-      <c r="B180" s="22"/>
+      <c r="B180" s="23"/>
       <c r="C180" s="6" t="s">
         <v>281</v>
       </c>
@@ -13378,7 +13378,7 @@
       <c r="A181" s="6">
         <v>180</v>
       </c>
-      <c r="B181" s="22"/>
+      <c r="B181" s="23"/>
       <c r="C181" s="6" t="s">
         <v>282</v>
       </c>
@@ -13444,7 +13444,7 @@
       <c r="A182" s="6">
         <v>181</v>
       </c>
-      <c r="B182" s="22"/>
+      <c r="B182" s="23"/>
       <c r="C182" s="6" t="s">
         <v>283</v>
       </c>
@@ -13510,7 +13510,7 @@
       <c r="A183" s="6">
         <v>182</v>
       </c>
-      <c r="B183" s="22"/>
+      <c r="B183" s="23"/>
       <c r="C183" s="6" t="s">
         <v>284</v>
       </c>
@@ -13576,11 +13576,11 @@
       <c r="A184" s="6">
         <v>183</v>
       </c>
-      <c r="B184" s="22" t="s">
-        <v>291</v>
+      <c r="B184" s="23" t="s">
+        <v>295</v>
       </c>
       <c r="C184" s="7" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="D184" s="7" t="s">
         <v>130</v>
@@ -13644,9 +13644,9 @@
       <c r="A185" s="6">
         <v>184</v>
       </c>
-      <c r="B185" s="22"/>
+      <c r="B185" s="23"/>
       <c r="C185" s="7" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="D185" s="7" t="s">
         <v>130</v>
@@ -13710,9 +13710,9 @@
       <c r="A186" s="6">
         <v>185</v>
       </c>
-      <c r="B186" s="22"/>
+      <c r="B186" s="23"/>
       <c r="C186" s="7" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="D186" s="7" t="s">
         <v>130</v>
@@ -13776,9 +13776,9 @@
       <c r="A187" s="6">
         <v>186</v>
       </c>
-      <c r="B187" s="22"/>
+      <c r="B187" s="23"/>
       <c r="C187" s="7" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="D187" s="7" t="s">
         <v>130</v>
@@ -13842,9 +13842,9 @@
       <c r="A188" s="6">
         <v>187</v>
       </c>
-      <c r="B188" s="22"/>
+      <c r="B188" s="23"/>
       <c r="C188" s="7" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="D188" s="7" t="s">
         <v>130</v>
@@ -13908,7 +13908,7 @@
       <c r="A189" s="6">
         <v>188</v>
       </c>
-      <c r="B189" s="22" t="s">
+      <c r="B189" s="23" t="s">
         <v>212</v>
       </c>
       <c r="C189" s="6" t="s">
@@ -13976,7 +13976,7 @@
       <c r="A190" s="6">
         <v>189</v>
       </c>
-      <c r="B190" s="22"/>
+      <c r="B190" s="23"/>
       <c r="C190" s="6" t="s">
         <v>92</v>
       </c>
@@ -14042,7 +14042,7 @@
       <c r="A191" s="6">
         <v>190</v>
       </c>
-      <c r="B191" s="22"/>
+      <c r="B191" s="23"/>
       <c r="C191" s="6" t="s">
         <v>93</v>
       </c>
@@ -14108,7 +14108,7 @@
       <c r="A192" s="6">
         <v>191</v>
       </c>
-      <c r="B192" s="22"/>
+      <c r="B192" s="23"/>
       <c r="C192" s="6" t="s">
         <v>94</v>
       </c>
@@ -14174,7 +14174,7 @@
       <c r="A193" s="6">
         <v>192</v>
       </c>
-      <c r="B193" s="22" t="s">
+      <c r="B193" s="23" t="s">
         <v>213</v>
       </c>
       <c r="C193" s="6" t="s">
@@ -14242,7 +14242,7 @@
       <c r="A194" s="6">
         <v>193</v>
       </c>
-      <c r="B194" s="22"/>
+      <c r="B194" s="23"/>
       <c r="C194" s="6" t="s">
         <v>96</v>
       </c>
@@ -14512,7 +14512,7 @@
       <c r="A198" s="6">
         <v>197</v>
       </c>
-      <c r="B198" s="22" t="s">
+      <c r="B198" s="23" t="s">
         <v>220</v>
       </c>
       <c r="C198" s="6" t="s">
@@ -14580,7 +14580,7 @@
       <c r="A199" s="6">
         <v>198</v>
       </c>
-      <c r="B199" s="22"/>
+      <c r="B199" s="23"/>
       <c r="C199" s="6" t="s">
         <v>99</v>
       </c>
@@ -14646,7 +14646,7 @@
       <c r="A200" s="6">
         <v>199</v>
       </c>
-      <c r="B200" s="22"/>
+      <c r="B200" s="23"/>
       <c r="C200" s="6" t="s">
         <v>100</v>
       </c>
@@ -14712,7 +14712,7 @@
       <c r="A201" s="6">
         <v>200</v>
       </c>
-      <c r="B201" s="22"/>
+      <c r="B201" s="23"/>
       <c r="C201" s="6" t="s">
         <v>101</v>
       </c>
@@ -14778,7 +14778,7 @@
       <c r="A202" s="6">
         <v>201</v>
       </c>
-      <c r="B202" s="22" t="s">
+      <c r="B202" s="23" t="s">
         <v>214</v>
       </c>
       <c r="C202" s="6" t="s">
@@ -14846,7 +14846,7 @@
       <c r="A203" s="6">
         <v>202</v>
       </c>
-      <c r="B203" s="22"/>
+      <c r="B203" s="23"/>
       <c r="C203" s="6" t="s">
         <v>106</v>
       </c>
@@ -14912,7 +14912,7 @@
       <c r="A204" s="6">
         <v>203</v>
       </c>
-      <c r="B204" s="22"/>
+      <c r="B204" s="23"/>
       <c r="C204" s="6" t="s">
         <v>107</v>
       </c>
@@ -14978,7 +14978,7 @@
       <c r="A205" s="6">
         <v>204</v>
       </c>
-      <c r="B205" s="22"/>
+      <c r="B205" s="23"/>
       <c r="C205" s="6" t="s">
         <v>108</v>
       </c>
@@ -15044,7 +15044,7 @@
       <c r="A206" s="6">
         <v>205</v>
       </c>
-      <c r="B206" s="22"/>
+      <c r="B206" s="23"/>
       <c r="C206" s="6" t="s">
         <v>109</v>
       </c>
@@ -15110,7 +15110,7 @@
       <c r="A207" s="6">
         <v>206</v>
       </c>
-      <c r="B207" s="22"/>
+      <c r="B207" s="23"/>
       <c r="C207" s="6" t="s">
         <v>110</v>
       </c>
@@ -15176,7 +15176,7 @@
       <c r="A208" s="6">
         <v>207</v>
       </c>
-      <c r="B208" s="22"/>
+      <c r="B208" s="23"/>
       <c r="C208" s="6" t="s">
         <v>111</v>
       </c>
@@ -15242,7 +15242,7 @@
       <c r="A209" s="6">
         <v>208</v>
       </c>
-      <c r="B209" s="22"/>
+      <c r="B209" s="23"/>
       <c r="C209" s="6" t="s">
         <v>112</v>
       </c>
@@ -15308,7 +15308,7 @@
       <c r="A210" s="6">
         <v>209</v>
       </c>
-      <c r="B210" s="22"/>
+      <c r="B210" s="23"/>
       <c r="C210" s="6" t="s">
         <v>113</v>
       </c>
@@ -15374,7 +15374,7 @@
       <c r="A211" s="6">
         <v>210</v>
       </c>
-      <c r="B211" s="22"/>
+      <c r="B211" s="23"/>
       <c r="C211" s="6" t="s">
         <v>103</v>
       </c>
@@ -15440,7 +15440,7 @@
       <c r="A212" s="6">
         <v>211</v>
       </c>
-      <c r="B212" s="22"/>
+      <c r="B212" s="23"/>
       <c r="C212" s="6" t="s">
         <v>104</v>
       </c>
@@ -15506,7 +15506,7 @@
       <c r="A213" s="6">
         <v>212</v>
       </c>
-      <c r="B213" s="22"/>
+      <c r="B213" s="23"/>
       <c r="C213" s="6" t="s">
         <v>105</v>
       </c>
@@ -15572,7 +15572,7 @@
       <c r="A214" s="6">
         <v>213</v>
       </c>
-      <c r="B214" s="22" t="s">
+      <c r="B214" s="23" t="s">
         <v>254</v>
       </c>
       <c r="C214" s="6" t="s">
@@ -15640,7 +15640,7 @@
       <c r="A215" s="6">
         <v>214</v>
       </c>
-      <c r="B215" s="22"/>
+      <c r="B215" s="23"/>
       <c r="C215" s="6" t="s">
         <v>247</v>
       </c>
@@ -15706,7 +15706,7 @@
       <c r="A216" s="6">
         <v>215</v>
       </c>
-      <c r="B216" s="22"/>
+      <c r="B216" s="23"/>
       <c r="C216" s="6" t="s">
         <v>248</v>
       </c>
@@ -15772,7 +15772,7 @@
       <c r="A217" s="6">
         <v>216</v>
       </c>
-      <c r="B217" s="22"/>
+      <c r="B217" s="23"/>
       <c r="C217" s="6" t="s">
         <v>249</v>
       </c>
@@ -15838,7 +15838,7 @@
       <c r="A218" s="6">
         <v>217</v>
       </c>
-      <c r="B218" s="22"/>
+      <c r="B218" s="23"/>
       <c r="C218" s="6" t="s">
         <v>250</v>
       </c>
@@ -15904,7 +15904,7 @@
       <c r="A219" s="6">
         <v>218</v>
       </c>
-      <c r="B219" s="22"/>
+      <c r="B219" s="23"/>
       <c r="C219" s="6" t="s">
         <v>251</v>
       </c>
@@ -15970,7 +15970,7 @@
       <c r="A220" s="6">
         <v>219</v>
       </c>
-      <c r="B220" s="22"/>
+      <c r="B220" s="23"/>
       <c r="C220" s="6" t="s">
         <v>252</v>
       </c>
@@ -16036,7 +16036,7 @@
       <c r="A221" s="6">
         <v>220</v>
       </c>
-      <c r="B221" s="22"/>
+      <c r="B221" s="23"/>
       <c r="C221" s="6" t="s">
         <v>253</v>
       </c>
@@ -16129,6 +16129,38 @@
   </sheetData>
   <autoFilter ref="A1:V221" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <mergeCells count="48">
+    <mergeCell ref="B214:B221"/>
+    <mergeCell ref="B198:B201"/>
+    <mergeCell ref="B202:B213"/>
+    <mergeCell ref="B152:B154"/>
+    <mergeCell ref="B147:B151"/>
+    <mergeCell ref="B155:B161"/>
+    <mergeCell ref="B170:B172"/>
+    <mergeCell ref="B163:B169"/>
+    <mergeCell ref="B189:B192"/>
+    <mergeCell ref="B193:B194"/>
+    <mergeCell ref="B173:B177"/>
+    <mergeCell ref="B178:B183"/>
+    <mergeCell ref="B184:B188"/>
+    <mergeCell ref="B126:B131"/>
+    <mergeCell ref="B38:B39"/>
+    <mergeCell ref="B141:B146"/>
+    <mergeCell ref="B96:B98"/>
+    <mergeCell ref="B86:B89"/>
+    <mergeCell ref="B134:B138"/>
+    <mergeCell ref="B139:B140"/>
+    <mergeCell ref="B99:B102"/>
+    <mergeCell ref="B105:B107"/>
+    <mergeCell ref="B90:B95"/>
+    <mergeCell ref="B108:B111"/>
+    <mergeCell ref="B112:B113"/>
+    <mergeCell ref="B114:B117"/>
+    <mergeCell ref="B118:B125"/>
+    <mergeCell ref="B8:B9"/>
+    <mergeCell ref="B10:B15"/>
+    <mergeCell ref="B16:B17"/>
+    <mergeCell ref="B18:B19"/>
+    <mergeCell ref="B20:B27"/>
     <mergeCell ref="B28:B29"/>
     <mergeCell ref="B103:B104"/>
     <mergeCell ref="B2:B3"/>
@@ -16145,38 +16177,6 @@
     <mergeCell ref="B49:B51"/>
     <mergeCell ref="B52:B58"/>
     <mergeCell ref="B59:B61"/>
-    <mergeCell ref="B8:B9"/>
-    <mergeCell ref="B10:B15"/>
-    <mergeCell ref="B16:B17"/>
-    <mergeCell ref="B18:B19"/>
-    <mergeCell ref="B20:B27"/>
-    <mergeCell ref="B126:B131"/>
-    <mergeCell ref="B38:B39"/>
-    <mergeCell ref="B141:B146"/>
-    <mergeCell ref="B96:B98"/>
-    <mergeCell ref="B86:B89"/>
-    <mergeCell ref="B134:B138"/>
-    <mergeCell ref="B139:B140"/>
-    <mergeCell ref="B99:B102"/>
-    <mergeCell ref="B105:B107"/>
-    <mergeCell ref="B90:B95"/>
-    <mergeCell ref="B108:B111"/>
-    <mergeCell ref="B112:B113"/>
-    <mergeCell ref="B114:B117"/>
-    <mergeCell ref="B118:B125"/>
-    <mergeCell ref="B214:B221"/>
-    <mergeCell ref="B198:B201"/>
-    <mergeCell ref="B202:B213"/>
-    <mergeCell ref="B152:B154"/>
-    <mergeCell ref="B147:B151"/>
-    <mergeCell ref="B155:B161"/>
-    <mergeCell ref="B170:B172"/>
-    <mergeCell ref="B163:B169"/>
-    <mergeCell ref="B189:B192"/>
-    <mergeCell ref="B193:B194"/>
-    <mergeCell ref="B173:B177"/>
-    <mergeCell ref="B178:B183"/>
-    <mergeCell ref="B184:B188"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>